<commit_message>
Updated data to only 2020
</commit_message>
<xml_diff>
--- a/pandemic-loss-modeling/data/epidemics_marani_240816.xlsx
+++ b/pandemic-loss-modeling/data/epidemics_marani_240816.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lichong/Desktop/RA 23F Epidemic/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lichong/Documents/GitHub/pandemic-loss-modeling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2295CB99-6C51-4040-B16A-D8FC83BA3A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B064693-7C84-1F48-A10F-EEEDEE732B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="500" windowWidth="22620" windowHeight="14420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2183" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2179" uniqueCount="430">
   <si>
     <t>location</t>
   </si>
@@ -1677,7 +1677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O543"/>
+  <dimension ref="A1:O542"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -27154,53 +27154,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="543" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A543" t="s">
-        <v>38</v>
-      </c>
-      <c r="B543">
-        <v>2023</v>
-      </c>
-      <c r="C543">
-        <v>2023</v>
-      </c>
-      <c r="D543">
-        <v>1</v>
-      </c>
-      <c r="E543">
-        <v>4</v>
-      </c>
-      <c r="F543">
-        <v>8020000</v>
-      </c>
-      <c r="G543">
-        <v>4.9875311720698251E-4</v>
-      </c>
-      <c r="H543">
-        <v>4.9875311720698253E-3</v>
-      </c>
-      <c r="I543" t="s">
-        <v>382</v>
-      </c>
-      <c r="J543" t="s">
-        <v>402</v>
-      </c>
-      <c r="K543" t="s">
-        <v>415</v>
-      </c>
-      <c r="L543">
-        <v>1</v>
-      </c>
-      <c r="M543">
-        <v>0</v>
-      </c>
-      <c r="N543">
-        <v>1</v>
-      </c>
-      <c r="O543">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>